<commit_message>
refactor(backend): adaptar API para Calculadora Judicial e SQLite
Renomeia core.dttuser para core.users e atualiza imports, schemas, permissoes e autenticacao. Substitui referencias corporativas nos comparativos, templates, traducoes e extrato contabil.

Padroniza SQLite em todos os ambientes, parametriza hosts e SSO, atualiza dependencias e ajusta rotas, arquivos estaticos e inicializacao do Celery.
</commit_message>
<xml_diff>
--- a/backend/templates/EXTRATOCONTABIL.xlsx
+++ b/backend/templates/EXTRATOCONTABIL.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\waoliveira\Documents\DJUD\backend\uploads\juca\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\waoliveira\Documents\DJUD\backend\uploads\Calculadora Judicial\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDCD6EE-0DB4-4AC9-95D4-9AB13ACE75C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Ficha de Análise" sheetId="56" r:id="rId1"/>
     <sheet name="Extrato Contábil" sheetId="32" r:id="rId2"/>
-    <sheet name="JUCA=Calculation" sheetId="58" r:id="rId3"/>
+    <sheet name="CALCULADORA_JUDICIAL=Calculation" sheetId="58" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_285_13">#REF!</definedName>
@@ -257,31 +257,31 @@
     <t>Executor:</t>
   </si>
   <si>
-    <t>JUCALST=Premises</t>
-  </si>
-  <si>
-    <t>JUCALST=Sheets</t>
-  </si>
-  <si>
-    <t>JUCALST=Claim_Lawyer</t>
-  </si>
-  <si>
-    <t>JUCALST=Claim_Creditor</t>
-  </si>
-  <si>
-    <t>JUCALST=NoticeAJ</t>
-  </si>
-  <si>
-    <t>JUCALST=NoticeAJ_Vert</t>
-  </si>
-  <si>
-    <t>JUCALST=Claim_Creditor_Vert</t>
-  </si>
-  <si>
-    <t>JUCALST=Claim_Lawyer_Vert</t>
-  </si>
-  <si>
-    <t>JUCALST=FundDocument</t>
+    <t>CALCULADORA_JUDICIAL_LST=Premises</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=Sheets</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=Claim_Lawyer</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=Claim_Creditor</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=NoticeAJ</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=NoticeAJ_Vert</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=Claim_Creditor_Vert</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=Claim_Lawyer_Vert</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_LST=FundDocument</t>
   </si>
   <si>
     <t>Correção monetária</t>
@@ -323,85 +323,85 @@
     <t>Valor devido (BRL)</t>
   </si>
   <si>
-    <t>JUCA=process_number</t>
-  </si>
-  <si>
-    <t>JUCA=has_edital</t>
-  </si>
-  <si>
-    <t>JUCA=legal_number</t>
-  </si>
-  <si>
-    <t>JUCA=recovering_name</t>
-  </si>
-  <si>
-    <t>JUCA=has_advocative_hours</t>
-  </si>
-  <si>
-    <t>JUCA=date_rj_request</t>
-  </si>
-  <si>
-    <t>JUCA=admission</t>
-  </si>
-  <si>
-    <t>JUCA=dismissal</t>
-  </si>
-  <si>
-    <t>JUCA=date_rj_filing</t>
-  </si>
-  <si>
-    <t>JUCA=date_citation</t>
-  </si>
-  <si>
-    <t>JUCA=default_interest</t>
-  </si>
-  <si>
-    <t>JUCA=advocative_hours</t>
-  </si>
-  <si>
-    <t>JUCA=executor</t>
-  </si>
-  <si>
-    <t>JUCA=reviewer</t>
-  </si>
-  <si>
-    <t>JUCA=approver</t>
-  </si>
-  <si>
-    <t>JUCA=court_name</t>
-  </si>
-  <si>
-    <t>Recuperanda JUCA=recovering_name</t>
-  </si>
-  <si>
-    <t>JUCA=fine</t>
-  </si>
-  <si>
-    <t>Incidente Nº JUCA=incident_number</t>
-  </si>
-  <si>
-    <t>JUCA=credor_name</t>
-  </si>
-  <si>
-    <t>Ficha de Análise de  JUCA=credor_name</t>
-  </si>
-  <si>
-    <t>Credor (a) :  JUCA=credor_name</t>
-  </si>
-  <si>
-    <t>JUCA=legend_monetary_correction_update</t>
+    <t>CALCULADORA_JUDICIAL=process_number</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=has_edital</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=legal_number</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=recovering_name</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=has_advocative_hours</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=date_rj_request</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=admission</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=dismissal</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=date_rj_filing</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=date_citation</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=default_interest</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=advocative_hours</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=executor</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=reviewer</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=approver</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=court_name</t>
+  </si>
+  <si>
+    <t>Recuperanda CALCULADORA_JUDICIAL=recovering_name</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=fine</t>
+  </si>
+  <si>
+    <t>Incidente Nº CALCULADORA_JUDICIAL=incident_number</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=credor_name</t>
+  </si>
+  <si>
+    <t>Ficha de Análise de  CALCULADORA_JUDICIAL=credor_name</t>
+  </si>
+  <si>
+    <t>Credor (a) :  CALCULADORA_JUDICIAL=credor_name</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=legend_monetary_correction_update</t>
   </si>
   <si>
     <t>Informações da solicitação do credor</t>
   </si>
   <si>
-    <t>DEMONSTRATIVO DE CÁLCULO NOS AUTOS DA RECUPERAÇÃO JUDICIAL DE JUCA=recovering_name JUCA=court_name</t>
-  </si>
-  <si>
-    <t>JUCA=index_name</t>
-  </si>
-  <si>
-    <t>JUCA=legend_citation_filling</t>
+    <t>DEMONSTRATIVO DE CÁLCULO NOS AUTOS DA RECUPERAÇÃO JUDICIAL DE CALCULADORA_JUDICIAL=recovering_name CALCULADORA_JUDICIAL=court_name</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=index_name</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL=legend_citation_filling</t>
   </si>
   <si>
     <t>Premissas:</t>
@@ -419,13 +419,13 @@
     <t>Descrição</t>
   </si>
   <si>
-    <t>JUCAD=legend_default_interest</t>
-  </si>
-  <si>
-    <t>JUCAD=legend_fine</t>
-  </si>
-  <si>
-    <t>JUCAD=legend_advocative_hours</t>
+    <t>CALCULADORA_JUDICIAL_D=legend_default_interest</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_D=legend_fine</t>
+  </si>
+  <si>
+    <t>CALCULADORA_JUDICIAL_D=legend_advocative_hours</t>
   </si>
 </sst>
 </file>

</xml_diff>